<commit_message>
update NT database: remove old papers and update metadata
</commit_message>
<xml_diff>
--- a/论文处理信息登记表.xlsx
+++ b/论文处理信息登记表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rockie\Desktop\大创\Date Record\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE730BE-6EB7-4F8E-AFEB-9F827A848755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8CE1E5C-2A5F-4138-999F-413BEFFA33D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="451" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="58">
   <si>
     <t>Paper 数据登记表</t>
   </si>
@@ -205,6 +205,14 @@
   </si>
   <si>
     <t>刘芸琪</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>待复审</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>通过</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -648,15 +656,17 @@
         <v>16</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="3"/>
+      <c r="H5" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="J5" s="1" t="s">
         <v>20</v>
       </c>
@@ -678,21 +688,22 @@
         <v>17</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="J6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="K6" s="1">
-        <f>COUNTIF(E5:E976,"是")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="25.5" customHeight="1">
@@ -973,7 +984,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>18</v>
@@ -981,7 +992,9 @@
       <c r="G18" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H18" s="3"/>
+      <c r="H18" s="3" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="25.5" customHeight="1">
       <c r="A19" s="5" t="s">

</xml_diff>

<commit_message>
update 03_PROFILES: 修改登记表update check_result
</commit_message>
<xml_diff>
--- a/论文处理信息登记表.xlsx
+++ b/论文处理信息登记表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rockie\Desktop\大创\Date Record\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0A9485-A755-4E51-9D87-80BED38B4988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63611F78-5B2C-4EF1-B7F3-B4FBD72B3714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="451" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="69">
   <si>
     <t>Paper 数据登记表</t>
   </si>
@@ -745,8 +745,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="1">
-        <f>COUNTIF(E5:E974,"是")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="25.5" customHeight="1">
@@ -1175,15 +1174,17 @@
         <v>17</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H24" s="3"/>
+      <c r="H24" s="3" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="25.5" customHeight="1">
       <c r="A25" s="5" t="s">

</xml_diff>

<commit_message>
update NT database: 修改登记表和数据
</commit_message>
<xml_diff>
--- a/论文处理信息登记表.xlsx
+++ b/论文处理信息登记表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rockie\Desktop\大创\Date Record\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63611F78-5B2C-4EF1-B7F3-B4FBD72B3714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50799B7D-7F9F-45C4-A997-B96B11062BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="451" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="69">
   <si>
     <t>Paper 数据登记表</t>
   </si>
@@ -745,7 +745,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="25.5" customHeight="1">
@@ -1608,15 +1608,17 @@
         <v>52</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H42" s="3"/>
+      <c r="H42" s="3" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="43" spans="1:8" ht="25.5" customHeight="1">
       <c r="A43" s="5" t="s">

</xml_diff>